<commit_message>
fixed eight GC testcases
</commit_message>
<xml_diff>
--- a/InputFiles/GC/TC01_GC_phs001524_Gender-Male_ExperimentStrat-DNASeq.xlsx
+++ b/InputFiles/GC/TC01_GC_phs001524_Gender-Male_ExperimentStrat-DNASeq.xlsx
@@ -516,9 +516,10 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (p:participant)-[:of_study]-&gt;(s:study)
+          <t>MATCH (f:file)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
 WHERE s.phs_accession = "phs001524"
   AND p.sex = "Male"
+  AND f.experimental_strategy_and_data_subtypes CONTAINS "DNA-Seq"
 WITH DISTINCT p, s
 OPTIONAL MATCH (samp_all:sample)-[:of_participant]-&gt;(p)
 WITH p, s, samp_all
@@ -537,23 +538,21 @@
   p.sex AS sex,
   samples
 ORDER BY p.participant_id ASC
-LIMIT 100
-</t>
+LIMIT 100</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (p:participant)-[:of_study]-&gt;(s:study)
+          <t>MATCH (f:file)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
 WHERE s.phs_accession = "phs001524"
   AND p.sex = "Male"
-OPTIONAL MATCH (samp:sample)-[:of_participant]-&gt;(p)
-OPTIONAL MATCH (f:file)-[:of_participant]-&gt;(p)
+  AND f.experimental_strategy_and_data_subtypes CONTAINS "DNA-Seq"
+OPTIONAL MATCH (f)-[:from_sample]-&gt;(samp:sample)
 RETURN
   count(DISTINCT s) AS Studies,
   count(DISTINCT p) AS Participants,
   count(DISTINCT samp) AS Samples,
-  count(DISTINCT f) AS Files
-</t>
+  count(DISTINCT f) AS Files</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -575,18 +574,18 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+          <t>MATCH (f:file)-[:from_sample]-&gt;(samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
 WHERE s.phs_accession = "phs001524"
   AND p.sex = "Male"
-RETURN
+  AND f.experimental_strategy_and_data_subtypes CONTAINS "DNA-Seq"
+RETURN DISTINCT
   s.study_acronym AS study_name,
   s.phs_accession AS accession,
   samp.sample_id AS sample_id,
   COALESCE(samp.sample_name, samp.sample_id) AS sample_name,
   COALESCE(samp.Organization_Name, "Not specified in data") AS organization_name
 ORDER BY samp.sample_id ASC
-LIMIT 100
-</t>
+LIMIT 100</t>
         </is>
       </c>
       <c r="C3" s="2" t="n"/>
@@ -599,11 +598,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (f:file)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+          <t>MATCH (f:file)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
 WHERE s.phs_accession = "phs001524"
   AND p.sex = "Male"
+  AND f.experimental_strategy_and_data_subtypes CONTAINS "DNA-Seq"
 OPTIONAL MATCH (f)-[:from_sample]-&gt;(samp:sample)
-RETURN
+RETURN DISTINCT
   s.study_name AS study_name,
   s.phs_accession AS accession,
   f.file_name AS file_name,
@@ -611,8 +611,7 @@
   f.file_type AS file_type,
   COALESCE(samp.sample_id, "Not Applicable") AS sample_id
 ORDER BY f.file_name ASC
-LIMIT 100
-</t>
+LIMIT 100</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>

</xml_diff>